<commit_message>
updates with DADA2 output with every plate from SDZWA + Sophie's Wild Orca + NOAA's samples
</commit_message>
<xml_diff>
--- a/metadata/Plate1/SRKW_Diet_Plate1_MetaData.xlsx
+++ b/metadata/Plate1/SRKW_Diet_Plate1_MetaData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/endouser/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/mball3_uw_edu/Documents/Documents/WADE LAB/SRKW/metadata/Plate1/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A7ED62-0B80-4F43-9E6C-92B8F0CF2FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="500" windowWidth="26560" windowHeight="16020" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
+    <workbookView xWindow="27250" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -722,13 +722,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A0E5F67-981F-2842-8BC9-09C804A53EC3}">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="2" max="2" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.8125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -751,7 +751,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -774,7 +774,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -820,7 +820,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -843,7 +843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -866,7 +866,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -889,7 +889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -912,7 +912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -935,7 +935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -958,7 +958,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -981,7 +981,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1533,7 +1533,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1556,7 +1556,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A47">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
Updates code to better match seqtab.nochim rownames to metadata rownames; still need to add in Amy and Sophia's samples
</commit_message>
<xml_diff>
--- a/metadata/Plate1/SRKW_Diet_Plate1_MetaData.xlsx
+++ b/metadata/Plate1/SRKW_Diet_Plate1_MetaData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/mball3_uw_edu/Documents/Documents/WADE LAB/SRKW/metadata/Plate1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A7ED62-0B80-4F43-9E6C-92B8F0CF2FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{86A7ED62-0B80-4F43-9E6C-92B8F0CF2FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C5EBE1A-E515-4FF3-AD26-DB516CD9D956}"/>
   <bookViews>
-    <workbookView xWindow="27250" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{518B7A33-C5FE-E642-B8D5-47A99A98280E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -753,94 +753,94 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E2">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="G2">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
+        <v>25</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
         <v>54</v>
       </c>
       <c r="E3">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G3">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A4">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>52</v>
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E4">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G4">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A5">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
         <v>54</v>
       </c>
       <c r="E5">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="G5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.5">
@@ -868,13 +868,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A7">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
+        <v>29</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D7" t="s">
         <v>54</v>
@@ -883,412 +883,412 @@
         <v>2023</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A8">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
         <v>54</v>
       </c>
       <c r="E8">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
         <v>54</v>
       </c>
       <c r="E9">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="F9" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A10">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
         <v>54</v>
       </c>
       <c r="E10">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="G10">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A11">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E11">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="F11" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="G11">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="D12" t="s">
         <v>54</v>
       </c>
       <c r="E12">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G12">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>16</v>
+        <v>36</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E13">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G13">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A14">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
         <v>54</v>
       </c>
       <c r="E14">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
       <c r="G14">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" t="s">
-        <v>60</v>
+        <v>3</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D15" t="s">
         <v>54</v>
       </c>
       <c r="E15">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>19</v>
+        <v>4</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D16" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E16">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A17">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" t="s">
-        <v>63</v>
+        <v>50</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E17">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F17" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A18">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" t="s">
-        <v>65</v>
+        <v>51</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E18">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="G18">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A19">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E19">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F19" t="s">
         <v>83</v>
       </c>
       <c r="G19">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A20">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D20" t="s">
         <v>54</v>
       </c>
       <c r="E20">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G20">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>24</v>
+        <v>34</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D21" t="s">
         <v>54</v>
       </c>
       <c r="E21">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F21" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G21">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>25</v>
+        <v>32</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E22">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F22" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G22">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A23">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D23" t="s">
         <v>54</v>
       </c>
       <c r="E23">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F23" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G23">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A24">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E24">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G24">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A25">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>52</v>
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>59</v>
       </c>
       <c r="D25" t="s">
         <v>54</v>
@@ -1297,67 +1297,67 @@
         <v>2023</v>
       </c>
       <c r="F25" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G25">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" t="s">
-        <v>64</v>
+        <v>40</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="D26" t="s">
         <v>54</v>
       </c>
       <c r="E26">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="G26">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" s="5" t="s">
         <v>31</v>
       </c>
+      <c r="B27" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E27">
         <v>2024</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A28">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D28" t="s">
         <v>79</v>
@@ -1366,18 +1366,18 @@
         <v>2024</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G28">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A29">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C29" t="s">
         <v>69</v>
@@ -1389,24 +1389,24 @@
         <v>2024</v>
       </c>
       <c r="F29" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G29">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A30">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D30" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E30">
         <v>2024</v>
@@ -1415,18 +1415,18 @@
         <v>82</v>
       </c>
       <c r="G30">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D31" t="s">
         <v>79</v>
@@ -1435,21 +1435,21 @@
         <v>2024</v>
       </c>
       <c r="F31" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G31">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>36</v>
+        <v>14</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D32" t="s">
         <v>54</v>
@@ -1458,30 +1458,30 @@
         <v>2024</v>
       </c>
       <c r="F32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G32">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A33">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D33" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E33">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F33" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G33">
         <v>1</v>
@@ -1489,255 +1489,255 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A34">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="C34" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D34" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E34">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G34">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A35">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="D35" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E35">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G35">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>40</v>
+        <v>12</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="D36" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E36">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F36" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G36">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C37" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="D37" t="s">
         <v>54</v>
       </c>
       <c r="E37">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F37" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G37">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A38">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D38" t="s">
         <v>54</v>
       </c>
       <c r="E38">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G38">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A39">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="C39" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D39" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E39">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="F39" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="G39">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A40">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="D40" t="s">
         <v>54</v>
       </c>
       <c r="E40">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="F40" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="G40">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>52</v>
+        <v>21</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" t="s">
+        <v>67</v>
       </c>
       <c r="D41" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="E41">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F41" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="G41">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>52</v>
+        <v>20</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" t="s">
+        <v>67</v>
       </c>
       <c r="D42" t="s">
         <v>54</v>
       </c>
       <c r="E42">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="F42" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G42">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A43">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="C43" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D43" t="s">
         <v>54</v>
       </c>
       <c r="E43">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="F43" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="G43">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A44">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>52</v>
-      </c>
-      <c r="E44" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="E44">
+        <v>2022</v>
       </c>
       <c r="F44" t="s">
-        <v>52</v>
-      </c>
-      <c r="G44" t="s">
-        <v>52</v>
+        <v>85</v>
+      </c>
+      <c r="G44">
+        <v>22</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.5">
@@ -1765,33 +1765,33 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A46">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C46" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" t="s">
+        <v>77</v>
+      </c>
+      <c r="D46" t="s">
         <v>52</v>
       </c>
-      <c r="D46" t="s">
-        <v>54</v>
-      </c>
-      <c r="E46">
-        <v>2022</v>
+      <c r="E46" t="s">
+        <v>52</v>
       </c>
       <c r="F46" t="s">
-        <v>55</v>
-      </c>
-      <c r="G46">
-        <v>6</v>
+        <v>52</v>
+      </c>
+      <c r="G46" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A47">
+        <v>41</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>52</v>
@@ -1803,13 +1803,16 @@
         <v>2022</v>
       </c>
       <c r="F47" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="G47">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G47">
+    <sortCondition ref="B2:B47"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>